<commit_message>
Exercise original payroll and ordinary account totals with retained identity-safe sources
</commit_message>
<xml_diff>
--- a/fixtures/adaptive-planning/sheet-export.xlsx
+++ b/fixtures/adaptive-planning/sheet-export.xlsx
@@ -125,7 +125,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>synthetic-easel-4</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -135,12 +135,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>synthetic-easel-70</t>
+          <t>Alex Morgan</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>synthetic-easel-80</t>
+          <t>Principal engineer</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -232,7 +232,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>synthetic-easel-4</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -242,12 +242,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>synthetic-easel-71</t>
+          <t>Jordan Lee</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>synthetic-easel-81</t>
+          <t>Financial analyst</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -339,7 +339,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>synthetic-easel-4</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -349,12 +349,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>synthetic-easel-72</t>
+          <t>Taylor Reed</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>synthetic-easel-82</t>
+          <t>Support specialist</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -446,7 +446,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>synthetic-easel-4</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -461,7 +461,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>synthetic-easel-83</t>
+          <t>Planned engineer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>synthetic-easel-4</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>synthetic-easel-84</t>
+          <t>Planned analyst</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">

</xml_diff>